<commit_message>
docs: mark the FedEx rate table as current
Kai confirmed the rate card is the one in force. The PDF carries no
effective date of its own, so the workbook now records who confirmed it
and when, alongside a note to update that line whenever FedEx sends a
replacement — the sheet should never again be in a state where its
currency is unknowable from the file itself.

Also states plainly that the table has no origin or zone dimension: one
national rate regardless of which facility ships. That was an open
question when reading the card and it changes nothing in the lookup, but
it belongs on the record rather than in a chat message.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RFdtYaoBaVuFihSh1Mu5xS
</commit_message>
<xml_diff>
--- a/docs/data/fedex-shipping-rates.xlsx
+++ b/docs/data/fedex-shipping-rates.xlsx
@@ -4459,7 +4459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4485,145 +4485,169 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="26" customHeight="1">
       <c r="A4" s="27" t="inlineStr">
         <is>
+          <t>유효성</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>현재 유효한 표 — Kai 확인 2026-09-13. 문서 자체에는 발효일자 표기가 없으므로, FedEx가 새 요금표를 보내오면 Rate Table 시트를 갱신하고 이 줄의 날짜를 함께 고칠 것.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>적용 범위</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>출발 시설·존(zone) 구분 없는 단일 표. GA/NJ/TX/NV/CA 어디서 나가든 같은 요금으로 적용.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
           <t>전사 방법</t>
         </is>
       </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B6" s="28" t="inlineStr">
         <is>
           <t>PDF에 텍스트 레이어가 없어(글자가 전부 벡터 외곽선) 자동 추출 불가. 5배 렌더링 후 7개 밴드로 나눠 육안 전사, 이상 셀은 8~11배로 재확인.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>검증 1차</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B7" s="28" t="inlineStr">
         <is>
           <t>170칸 중 공란 3칸 제외 167개 값. Sat−1Day=$33.07 불변식이 34행 중 33행에서 성립, 전 열 단조 증가, 전 행 등급 순서 정상. Verification 시트에 수식으로 남김.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="27" t="inlineStr">
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>검증 2차</t>
         </is>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>1차 검사는 3-Day 컬럼을 단조성으로만 커버해 가장 약했음. 9배 렌더로 From·Ground·3-Day·2-Day를 1차와 별개로 다시 판독해 136셀 대조 — 불일치 0. 해당 컬럼 확정.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="27" t="inlineStr">
-        <is>
-          <t>수식 검증</t>
-        </is>
-      </c>
-      <c r="B7" s="28" t="inlineStr">
-        <is>
-          <t>942개 수식 셀 전체 평가, 오류 0. 파이썬 독립 계산과 표본 대조 일치. (LibreOffice가 이 환경에서 동작하지 않아 formulas 엔진으로 평가함)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>확인 필요 1</t>
+          <t>수식 검증</t>
         </is>
       </c>
       <c r="B9" s="28" t="inlineStr">
         <is>
-          <t>Ground 요금 공란 — $37.00~$52.00, $52.00~$74.00, $74.00~$98.00 세 구간. 무료배송인지 Ground 미제공인지? (Danny)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="27" t="inlineStr">
-        <is>
-          <t>확인 필요 2</t>
-        </is>
-      </c>
-      <c r="B10" s="28" t="inlineStr">
-        <is>
-          <t>$894.00–$968.00 구간 Sat-Overnight = $870.94. 규칙대로면 $780.94. 원본 오타 의심. (FedEx/Danny)</t>
+          <t>942개 수식 셀 전체 평가, 오류 0. 파이썬 독립 계산과 표본 대조 일치. (LibreOffice가 이 환경에서 동작하지 않아 formulas 엔진으로 평가함)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="27" t="inlineStr">
         <is>
+          <t>확인 필요 1</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>Ground 요금 공란 — $37.00~$52.00, $52.00~$74.00, $74.00~$98.00 세 구간. 무료배송인지 Ground 미제공인지? (Danny)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>확인 필요 2</t>
+        </is>
+      </c>
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>$894.00–$968.00 구간 Sat-Overnight = $870.94. 규칙대로면 $780.94. 원본 오타 의심. (FedEx/Danny)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
           <t>확인 필요 3</t>
         </is>
       </c>
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B13" s="28" t="inlineStr">
         <is>
           <t>구간 틈 2곳 — $98.00~$98.01, $521.00~$522.00. 경계 금액이 어느 구간인지. 이 파일은 'From ≤ 금액' 규칙으로 아래 구간에 흡수.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="27" t="inlineStr">
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>확정</t>
         </is>
       </c>
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B14" s="28" t="inlineStr">
         <is>
           <t>조회 기준 = 주문 subtotal (세금 전, 배송비 제외). Kai 확인 2026-09-10. 업그레이드 추가요금을 더해도 조회 구간이 바뀌지 않으므로 재계산 문제 없음.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="27" t="inlineStr">
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>자동화 제외</t>
         </is>
       </c>
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>NEXT DAY STANDARD / NEXT DAY EARLY 8:30AM — 원본에 'VARIES BY LOC.'로만 표기, 요금값 없음.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="27" t="inlineStr">
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>조건부</t>
         </is>
       </c>
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>SAT-OVERNIGHT — 원본 주석: 모든 도시에서 가능하지 않으니 결제 전 확인. Saturday 옵션은 금요일 Express 주문에만. Ground도 토요일 배송이 되는 경우가 있음.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="52" customHeight="1">
-      <c r="A17" s="27" t="inlineStr">
+    <row r="19" ht="52" customHeight="1">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>원본 주석</t>
         </is>
       </c>
-      <c r="B17" s="28" t="inlineStr">
+      <c r="B19" s="28" t="inlineStr">
         <is>
           <t>Ground shipping is not a guaranteed service, but once "In transit", FEDEX guarantees the package will arrive by the ETA on their site. So, we cannot guarantee when the package will arrive before it ships out, but we can state, once UPS provides an ETA, they guarantee it will deliver by that time.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="39" customHeight="1">
-      <c r="A18" s="27" t="inlineStr">
+    <row r="20" ht="39" customHeight="1">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>원본 주석</t>
         </is>
       </c>
-      <c r="B18" s="28" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>IMPORTANT NOTE: Saturday options is not available for all cities, please check before taking payment. Saturday Option is only available on Friday for Express orders. Ground shipping does deliver on Saturdays sometimes.</t>
         </is>

</xml_diff>